<commit_message>
separate vip2023, vip2025 week 6, logic tests and small fixes
</commit_message>
<xml_diff>
--- a/data/normalo2026.xlsx
+++ b/data/normalo2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/isabelhaas/Documents/Coding/aytogermany/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC404B9D-93AB-9947-A6FD-581B93CD1D17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A05C07E1-4AAF-E246-9569-DA90FD2006C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9740" yWindow="3560" windowWidth="32520" windowHeight="18420" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5880" yWindow="3560" windowWidth="32520" windowHeight="18420" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Candidates" sheetId="1" r:id="rId1"/>

</xml_diff>